<commit_message>
Create expense tracker with Excel storage and validation
</commit_message>
<xml_diff>
--- a/Day_20/Expense Tracker/Expense Tracker.xlsx
+++ b/Day_20/Expense Tracker/Expense Tracker.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Expense Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Expense Tracker" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +414,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,36 +460,136 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Travel</t>
+          <t>Te</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Going office</t>
+          <t>jhbf</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>31-12-2020</t>
+          <t>09-09-2023</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Party</t>
+          <t>hkgfds</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">New year celebration </t>
+          <t>ngfds</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>340</v>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>09-07-2024</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>hgfd</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ngfd</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>09-09-2023</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>fdsad</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>gfdsfad</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>09-08-2023</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>hjcgfdsadddhfd</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>gfhgmfdgsfaa</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>09-08-2034</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>gfndd</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>fdgsfa</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>09-08-2023</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>hgfdzfAD</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>bvcgfxdsz</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>